<commit_message>
included country and region HQ logic from Benjamin
</commit_message>
<xml_diff>
--- a/plot/storage/output/ongoing/ongoing_tech_filter_by_iso2_q.xlsx
+++ b/plot/storage/output/ongoing/ongoing_tech_filter_by_iso2_q.xlsx
@@ -571,7 +571,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>121616428.5714286</v>
+        <v>86616428.57142857</v>
       </c>
       <c r="H2" t="n">
         <v>9166666.666666666</v>
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>133074761.9047619</v>
+        <v>94185873.01587301</v>
       </c>
       <c r="H3" t="n">
         <v>9166666.666666666</v>
@@ -713,7 +713,7 @@
         <v>18333333.33333333</v>
       </c>
       <c r="G4" t="n">
-        <v>155991428.5714286</v>
+        <v>109324761.9047619</v>
       </c>
       <c r="H4" t="n">
         <v>9166666.666666666</v>
@@ -784,7 +784,7 @@
         <v>55000000</v>
       </c>
       <c r="G5" t="n">
-        <v>155991428.5714286</v>
+        <v>109324761.9047619</v>
       </c>
       <c r="H5" t="n">
         <v>21388888.88888889</v>
@@ -793,7 +793,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>12422222.22222222</v>
+        <v>5755555.555555555</v>
       </c>
       <c r="K5" t="n">
         <v>27500000</v>
@@ -855,7 +855,7 @@
         <v>55000000</v>
       </c>
       <c r="G6" t="n">
-        <v>100991428.5714286</v>
+        <v>89324761.90476191</v>
       </c>
       <c r="H6" t="n">
         <v>82500000</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>36866666.66666666</v>
+        <v>23533333.33333333</v>
       </c>
       <c r="K6" t="n">
         <v>18333333.33333333</v>
@@ -926,7 +926,7 @@
         <v>55000000</v>
       </c>
       <c r="G7" t="n">
-        <v>99991428.57142857</v>
+        <v>88324761.90476191</v>
       </c>
       <c r="H7" t="n">
         <v>82500000</v>
@@ -935,7 +935,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>36866666.66666666</v>
+        <v>23533333.33333333</v>
       </c>
       <c r="K7" t="n">
         <v>18333333.33333333</v>
@@ -997,7 +997,7 @@
         <v>57224255.83333333</v>
       </c>
       <c r="G8" t="n">
-        <v>119201984.1269841</v>
+        <v>107535317.4603175</v>
       </c>
       <c r="H8" t="n">
         <v>82500000</v>
@@ -1006,7 +1006,7 @@
         <v>3333333.333333333</v>
       </c>
       <c r="J8" t="n">
-        <v>36866666.66666666</v>
+        <v>23533333.33333333</v>
       </c>
       <c r="K8" t="n">
         <v>18333333.33333333</v>
@@ -1068,7 +1068,7 @@
         <v>61672767.49999999</v>
       </c>
       <c r="G9" t="n">
-        <v>269928884.7117795</v>
+        <v>258262218.0451128</v>
       </c>
       <c r="H9" t="n">
         <v>82500000</v>
@@ -1077,7 +1077,7 @@
         <v>10000000</v>
       </c>
       <c r="J9" t="n">
-        <v>59783333.33333333</v>
+        <v>27700000</v>
       </c>
       <c r="K9" t="n">
         <v>18333333.33333333</v>
@@ -1139,7 +1139,7 @@
         <v>61672767.49999999</v>
       </c>
       <c r="G10" t="n">
-        <v>298205827.0676692</v>
+        <v>286539160.4010025</v>
       </c>
       <c r="H10" t="n">
         <v>119166666.6666667</v>
@@ -1148,7 +1148,7 @@
         <v>10000000</v>
       </c>
       <c r="J10" t="n">
-        <v>105616666.6666667</v>
+        <v>36033333.33333333</v>
       </c>
       <c r="K10" t="n">
         <v>18333333.33333333</v>
@@ -1210,7 +1210,7 @@
         <v>68894989.72222221</v>
       </c>
       <c r="G11" t="n">
-        <v>291480628.6549708</v>
+        <v>279813961.9883041</v>
       </c>
       <c r="H11" t="n">
         <v>116111111.1111111</v>
@@ -1219,7 +1219,7 @@
         <v>10000000</v>
       </c>
       <c r="J11" t="n">
-        <v>105616666.6666667</v>
+        <v>36033333.33333333</v>
       </c>
       <c r="K11" t="n">
         <v>18333333.33333333</v>
@@ -1281,7 +1281,7 @@
         <v>102573916.9583333</v>
       </c>
       <c r="G12" t="n">
-        <v>313744517.5438597</v>
+        <v>302077850.877193</v>
       </c>
       <c r="H12" t="n">
         <v>110000000</v>
@@ -1290,7 +1290,7 @@
         <v>10000000</v>
       </c>
       <c r="J12" t="n">
-        <v>105616666.6666667</v>
+        <v>36033333.33333333</v>
       </c>
       <c r="K12" t="n">
         <v>18333333.33333333</v>
@@ -1352,7 +1352,7 @@
         <v>102573916.9583333</v>
       </c>
       <c r="G13" t="n">
-        <v>618054508.2067914</v>
+        <v>606387841.5401248</v>
       </c>
       <c r="H13" t="n">
         <v>110000000</v>
@@ -1361,7 +1361,7 @@
         <v>10000000</v>
       </c>
       <c r="J13" t="n">
-        <v>105616666.6666667</v>
+        <v>39366666.66666666</v>
       </c>
       <c r="K13" t="n">
         <v>12222222.22222222</v>
@@ -1423,7 +1423,7 @@
         <v>92551311.58333333</v>
       </c>
       <c r="G14" t="n">
-        <v>1388047415.626169</v>
+        <v>1376380748.959503</v>
       </c>
       <c r="H14" t="n">
         <v>110000000</v>
@@ -1432,7 +1432,7 @@
         <v>21111111.11111111</v>
       </c>
       <c r="J14" t="n">
-        <v>106727777.7777778</v>
+        <v>47144444.44444444</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1494,7 +1494,7 @@
         <v>72506100.83333333</v>
       </c>
       <c r="G15" t="n">
-        <v>1379888997.000438</v>
+        <v>1372111219.222661</v>
       </c>
       <c r="H15" t="n">
         <v>110000000</v>
@@ -1503,7 +1503,7 @@
         <v>43333333.33333334</v>
       </c>
       <c r="J15" t="n">
-        <v>108816666.6666667</v>
+        <v>49233333.33333333</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1574,7 +1574,7 @@
         <v>43333333.33333334</v>
       </c>
       <c r="J16" t="n">
-        <v>108750000</v>
+        <v>49166666.66666666</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1645,7 +1645,7 @@
         <v>43333333.33333334</v>
       </c>
       <c r="J17" t="n">
-        <v>108750000</v>
+        <v>46666666.66666666</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1716,7 +1716,7 @@
         <v>43333333.33333334</v>
       </c>
       <c r="J18" t="n">
-        <v>108750000</v>
+        <v>41666666.66666666</v>
       </c>
       <c r="K18" t="n">
         <v>147392290</v>
@@ -1787,7 +1787,7 @@
         <v>43333333.33333334</v>
       </c>
       <c r="J19" t="n">
-        <v>108750000</v>
+        <v>41666666.66666666</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -1858,7 +1858,7 @@
         <v>40000000</v>
       </c>
       <c r="J20" t="n">
-        <v>157638888.8888889</v>
+        <v>78333333.33333333</v>
       </c>
       <c r="K20" t="n">
         <v>32468305.63636363</v>
@@ -1929,7 +1929,7 @@
         <v>33333333.33333334</v>
       </c>
       <c r="J21" t="n">
-        <v>214166666.6666667</v>
+        <v>147500000</v>
       </c>
       <c r="K21" t="n">
         <v>91612761.38636363</v>
@@ -2000,7 +2000,7 @@
         <v>33333333.33333334</v>
       </c>
       <c r="J22" t="n">
-        <v>168333333.3333333</v>
+        <v>139166666.6666667</v>
       </c>
       <c r="K22" t="n">
         <v>91612761.38636363</v>
@@ -2071,7 +2071,7 @@
         <v>33333333.33333334</v>
       </c>
       <c r="J23" t="n">
-        <v>364487179.4871795</v>
+        <v>335320512.8205128</v>
       </c>
       <c r="K23" t="n">
         <v>81019159.50757575</v>
@@ -2142,7 +2142,7 @@
         <v>33333333.33333334</v>
       </c>
       <c r="J24" t="n">
-        <v>364487179.4871795</v>
+        <v>335320512.8205128</v>
       </c>
       <c r="K24" t="n">
         <v>99722848.30555555</v>
@@ -2213,7 +2213,7 @@
         <v>33333333.33333334</v>
       </c>
       <c r="J25" t="n">
-        <v>336153846.1538461</v>
+        <v>303653846.1538461</v>
       </c>
       <c r="K25" t="n">
         <v>125421300.0833333</v>
@@ -2284,7 +2284,7 @@
         <v>22222222.22222222</v>
       </c>
       <c r="J26" t="n">
-        <v>265876068.3760684</v>
+        <v>226709401.7094017</v>
       </c>
       <c r="K26" t="n">
         <v>127620574.4722222</v>
@@ -2355,7 +2355,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>172884615.3846154</v>
+        <v>133717948.7179487</v>
       </c>
       <c r="K27" t="n">
         <v>128720211.6666667</v>
@@ -2423,10 +2423,10 @@
         <v>681111111.111111</v>
       </c>
       <c r="I28" t="n">
-        <v>44444444.44444445</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>188340277.7777778</v>
+        <v>148638888.8888889</v>
       </c>
       <c r="K28" t="n">
         <v>128720211.6666667</v>
@@ -2494,10 +2494,10 @@
         <v>681111111.111111</v>
       </c>
       <c r="I29" t="n">
-        <v>66666666.66666667</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>342140716.374269</v>
+        <v>283036549.7076024</v>
       </c>
       <c r="K29" t="n">
         <v>128720211.6666667</v>
@@ -2565,10 +2565,10 @@
         <v>681111111.111111</v>
       </c>
       <c r="I30" t="n">
-        <v>66666666.66666667</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>449450657.8947369</v>
+        <v>347013157.8947368</v>
       </c>
       <c r="K30" t="n">
         <v>387479203.5555556</v>
@@ -2636,10 +2636,10 @@
         <v>837602339.1812865</v>
       </c>
       <c r="I31" t="n">
-        <v>66666666.66666667</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>466117324.5614035</v>
+        <v>363679824.5614035</v>
       </c>
       <c r="K31" t="n">
         <v>516858699.5000001</v>
@@ -2707,10 +2707,10 @@
         <v>922913336.5146199</v>
       </c>
       <c r="I32" t="n">
-        <v>66666666.66666667</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>398895102.3391813</v>
+        <v>363679824.5614035</v>
       </c>
       <c r="K32" t="n">
         <v>536170007.0833334</v>
@@ -2778,10 +2778,10 @@
         <v>922913336.5146199</v>
       </c>
       <c r="I33" t="n">
-        <v>66666666.66666667</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>365283991.2280702</v>
+        <v>363679824.5614035</v>
       </c>
       <c r="K33" t="n">
         <v>477025551.3333333</v>
@@ -2849,10 +2849,10 @@
         <v>907913336.5146199</v>
       </c>
       <c r="I34" t="n">
-        <v>66666666.66666667</v>
+        <v>22222222.22222222</v>
       </c>
       <c r="J34" t="n">
-        <v>365283991.2280702</v>
+        <v>363679824.5614035</v>
       </c>
       <c r="K34" t="n">
         <v>477025551.3333333</v>
@@ -2879,7 +2879,7 @@
         <v>39433383.76515152</v>
       </c>
       <c r="S34" t="n">
-        <v>19833333.33333333</v>
+        <v>130944444.4444444</v>
       </c>
       <c r="T34" t="n">
         <v>52500000</v>
@@ -2923,7 +2923,7 @@
         <v>66666666.66666667</v>
       </c>
       <c r="J35" t="n">
-        <v>301529605.2631579</v>
+        <v>299925438.5964912</v>
       </c>
       <c r="K35" t="n">
         <v>476796384.6666666</v>
@@ -2932,7 +2932,7 @@
         <v>8333333.333333334</v>
       </c>
       <c r="M35" t="n">
-        <v>1059502650.307315</v>
+        <v>1098391539.196204</v>
       </c>
       <c r="N35" t="n">
         <v>0</v>
@@ -2950,7 +2950,7 @@
         <v>32766717.09848485</v>
       </c>
       <c r="S35" t="n">
-        <v>65666666.66666666</v>
+        <v>232333333.3333333</v>
       </c>
       <c r="T35" t="n">
         <v>39722222.22222222</v>
@@ -2994,7 +2994,7 @@
         <v>66666666.66666667</v>
       </c>
       <c r="J36" t="n">
-        <v>44687500</v>
+        <v>43083333.33333333</v>
       </c>
       <c r="K36" t="n">
         <v>436447158.7777778</v>
@@ -3003,7 +3003,7 @@
         <v>2777777.777777778</v>
       </c>
       <c r="M36" t="n">
-        <v>1205462303.399321</v>
+        <v>1263795636.732655</v>
       </c>
       <c r="N36" t="n">
         <v>0</v>
@@ -3021,7 +3021,7 @@
         <v>7312171.643939395</v>
       </c>
       <c r="S36" t="n">
-        <v>65666666.66666666</v>
+        <v>232333333.3333333</v>
       </c>
       <c r="T36" t="n">
         <v>33333333.33333334</v>

</xml_diff>